<commit_message>
day 2 become day3, add new day 2
</commit_message>
<xml_diff>
--- a/AI_Program_Stage2.xlsx
+++ b/AI_Program_Stage2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mohammedbalkhair/Desktop/qasab-program/stage-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC0BE1E-BA71-A146-BD02-89BFB2AEEE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED40A852-BC69-E74A-B3BB-C10DD318C931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Lecture</t>
   </si>
@@ -51,15 +51,6 @@
 • Can describe hidden layers using the vision analogy
 • Can connect overfitting back to 'lazy nodes'
 • Can state 3 ways the brain analogy breaks down</t>
-  </si>
-  <si>
-    <t>By the end of this session, students can identify the genuine limits of current AI, explain why each limit exists from the inside, and think critically when an AI output sounds convincing.</t>
-  </si>
-  <si>
-    <t>• Can name and explain 4 genuine AI limits
-• Can explain WHY each limit exists, not just that it exists
-• Can apply the 'stochastic parrot' idea
-• Thinks critically before trusting a confident AI response</t>
   </si>
   <si>
     <t xml:space="preserve">QASAB Program — AI Stage 2 </t>
@@ -73,33 +64,6 @@
 Section 5 — Where The Analogy Breaks </t>
   </si>
   <si>
-    <t>Day 2
-Built in Our Image
-(مبني على صورتنا)</t>
-  </si>
-  <si>
-    <t>Day 3
-Where AI Falls Short
-(حيث يقصر الذكاء الاصطناعي)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Story: 'Yesterday we saw how AI was built to look like us. Today we find the cracks.'
-Section 1 — Opening Tension 
-Section 2 — Common Sense: The Invisible Knowledge Problem 
-Section 3 — Novelty: AI Cannot Figure Things Out 
-Section 4 — Hallucinations: The Deeper Why 
-Section 5 — The Accountability Gap 
-</t>
-  </si>
-  <si>
-    <t>S1: 'AI can beat chess champions — so what CAN'T it do?' → all limits share one root.
-S2: Common sense = knowledge from living. AI has text ABOUT the world, not experience OF it. 'I'm fine' ≠ fine — AI misses this.
-S3: Truly new situation → guesses nearest pattern. No 'aha' moment. No layer that wonders.
-S4: Only job = predict next token. No fact-checker. No 'I don't know.' Stochastic parrot: rearranging, not thinking.
-S5: No accountability. Wrong diagnosis/biased hiring/deepfake → who is responsible?
-- All limits share one root — AI has never lived.</t>
-  </si>
-  <si>
     <t>By the end of this session, students can explain why traditional logic fails at pattern recognition, identify the difference between data and engineered features, and manually manipulate weights to understand classical Machine Learning boundaries.</t>
   </si>
   <si>
@@ -110,25 +74,81 @@
 Section 4 — The Scaling Crisis (Bridge to Day 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">S1: You show a cat photo on the projector. You challenge the class to write strict "If-Else" rules to identify it. By flipping or shadowing the image, you prove that hardcoded pixel logic breaks down immediately.  
+    <t>Day 1
+(هندسة الأنماط)</t>
+  </si>
+  <si>
+    <t>S1: You show a cat photo on the projector. You challenge the class to write strict "If-Else" rules to identify it. By flipping or shadowing the image, you prove that hardcoded pixel logic breaks down immediately.  
 S2: Shifting from raw data to "Features." You map a complex silhouette on screen and guide the class to extract primitive geometries (lines, intersection points, aspect ratios).
 S3: Classical ML Mechanics. You display a basic linear formula on screen: 
 Score=(F1×W1)+(F2×W2)
 . You manually adjust sliders for the weights (W) on your screen to show how changing importance values shifts a basic classification line between data points, completely free of Deep Learning.
-S4: The Bridge. If a problem has millions of pixels, engineering these features and weights manually is impossible. Tomorrow, we look at how Deep Learning automates this using hidden layers inspired by the human brain. </t>
+S4: The Bridge. We just saw how hard it is to manually adjust just two weights. What if an image has millions of features? Doing this by hand is impossible. Tomorrow, we look at how the machine learns to adjust its own weights automatically.</t>
   </si>
   <si>
     <t>• Explains why rule-based programming fails at pattern recognition  
 • Differentiates between raw input data and engineered features
 • Understands how weights alter a classical machine learning prediction
-• Perfectly primed for the biological neuron and hidden layer analogies on Day 2</t>
-  </si>
-  <si>
-    <t>Day 1
-(هندسة الأنماط)</t>
-  </si>
-  <si>
-    <t>Day 4</t>
+• Realizes the mathematical necessity for automatic weight adjustment in Day 2</t>
+  </si>
+  <si>
+    <t>Day 3
+Built in Our Image
+(مبني على صورتنا)</t>
+  </si>
+  <si>
+    <t>Day 2
+The Learning Loop
+(دائرة التعلّم)</t>
+  </si>
+  <si>
+    <t>By the end of this session, students can explain the 4-step automated training cycle, understand how a machine measures its own mistakes, and visualize how it updates its weights without human intervention.</t>
+  </si>
+  <si>
+    <t>Story: 'Yesterday, we struggled to find the right weights by hand. Today, we give the machine a compass so it can find them on its own.'
+Section 1 — The Blind Guess
+Section 2 — Measuring the Error
+Section 3 — The Automatic Adjustment
+Section 4 — Bridge to the Brain (Day 3)</t>
+  </si>
+  <si>
+    <t>S1: The Start: The machine doesn't know anything, so it assigns completely random numbers to  W 1 and W 2 ​and makes a "Blind Guess."
+S2: The Error: The machine compares its blind guess to the actual correct answer in the training data. It calculates exactly "how wrong" it was.
+S3: The Loop: Introduce the circular training diagram. The machine uses a mathematical rule to nudge the weights up or down to reduce the error, then guesses again. It repeats this loop millions of times until the error is tiny.
+S4: The Bridge: This automatic loop works perfectly for flat numbers. But how do we structure these weights to recognize complex, layered things like faces? We need an architecture inspired by human biology.</t>
+  </si>
+  <si>
+    <t>Can outline the 4 steps of machine training: Guess, Measure, Adjust, Repeat
+• Understands that "learning" in AI is simply the mathematical reduction of error
+• Realizes that the machine does the exact same thing they did manually on Day 1, just millions of times faster
+• Primed for the Neural Network structure in Day 3</t>
+  </si>
+  <si>
+    <t>Day 4
+The Prompt Architect
+(مهندس الأوامر)</t>
+  </si>
+  <si>
+    <t>By the end of this session, students can design complex, structured prompts using established frameworks and successfully apply them across various generative AI interfaces to control the output.</t>
+  </si>
+  <si>
+    <t>Story: 'Now that we know exactly how the machine thinks and learns, let's learn how to speak its language perfectly to get exactly what we want.'
+Section 1 — The Art of the Instruction
+Section 2 — The RCTF Framework
+Section 3 — Advanced Constraints
+Section 4 — The Cross-Tool Application</t>
+  </si>
+  <si>
+    <t>Moves from casually chatting with AI to professionally engineering instructions
+• Memorizes and applies the RCTF framework
+• Understands how to force an AI to show its "chain of thought"
+• Realizes that prompt engineering is a universal skill that works across all generative platforms, regardless of the brand name</t>
+  </si>
+  <si>
+    <t>S1: Moving beyond "chatting." Explain that an AI is a powerful engine, but a weak prompt is a bad steering wheel. If you give a vague input, the AI's weights will generate a generic output.
+S2: Break down the RCTF Framework visually on screen: Role (Who is the AI?), Context (What is the background?), Task (What exactly needs to be done?), Format (How should it look?).
+S3: Teach advanced techniques: "Chain of Thought" (asking the AI to think step-by-step before answering) and setting strict negative constraints (telling it what not to do).
+S4: Live Demonstration. You take one perfectly structured prompt and apply it live to three different types of platforms: A text-generation model, an image-generation model, and an automated presentation-building model. You show how the exact same prompt engineering rules apply to all AI categories.</t>
   </si>
 </sst>
 </file>
@@ -568,7 +588,7 @@
     <row r="1" spans="2:6" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -594,63 +614,71 @@
     </row>
     <row r="4" spans="2:6" ht="183" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="219" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="213" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="222" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>